<commit_message>
Methane Modelle, Vergleichskript, Fehlerkorrektur Strompreis
Ersten Methane Modelle erstellt

Vergleichsskript an Methan angepasst

Strompreis in sechs modellen auf deutsche standorte angepasst
</commit_message>
<xml_diff>
--- a/Fischer_Tropsch/FischerTropsch_Naphta_Brownfield_Höchst/Datenbank.xlsx
+++ b/Fischer_Tropsch/FischerTropsch_Naphta_Brownfield_Höchst/Datenbank.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Fischer_Tropsch\FischerTropsch_Naphta_Brownfield_Südafrika\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Arbeit\06-FENES\09-P2X3\FENES_P2X\Fischer_Tropsch\FischerTropsch_Naphta_Brownfield_Höchst\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07363D30-605E-4ED4-B0B3-D2C2A3EDADA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73CA4FDD-00F8-4225-B93A-AA216170B769}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datenauswahl" sheetId="1" r:id="rId1"/>
@@ -1734,23 +1734,32 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1758,26 +1767,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1788,11 +1782,17 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3207,7 +3207,7 @@
         <v>75</v>
       </c>
       <c r="E55" s="3">
-        <v>9.2999999999999999E-2</v>
+        <v>0.1699</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>19</v>
@@ -3591,10 +3591,10 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="91" t="s">
+      <c r="A2" s="93" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="93" t="s">
+      <c r="B2" s="95" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="26" t="s">
@@ -3609,7 +3609,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="92"/>
+      <c r="A3" s="99"/>
       <c r="B3" s="89"/>
       <c r="C3" s="13" t="s">
         <v>107</v>
@@ -3623,7 +3623,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="92"/>
+      <c r="A4" s="99"/>
       <c r="B4" s="89"/>
       <c r="C4" s="13" t="s">
         <v>84</v>
@@ -3637,7 +3637,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="92"/>
+      <c r="A5" s="99"/>
       <c r="B5" s="89"/>
       <c r="C5" s="13" t="s">
         <v>138</v>
@@ -3651,7 +3651,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="92"/>
+      <c r="A6" s="99"/>
       <c r="B6" s="89"/>
       <c r="C6" s="13" t="s">
         <v>141</v>
@@ -3665,7 +3665,7 @@
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="92"/>
+      <c r="A7" s="99"/>
       <c r="B7" s="89"/>
       <c r="C7" s="13" t="s">
         <v>155</v>
@@ -3679,7 +3679,7 @@
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="92"/>
+      <c r="A8" s="99"/>
       <c r="B8" s="89"/>
       <c r="C8" s="13" t="s">
         <v>196</v>
@@ -3693,7 +3693,7 @@
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="92"/>
+      <c r="A9" s="99"/>
       <c r="B9" s="89"/>
       <c r="C9" s="13" t="s">
         <v>167</v>
@@ -3707,7 +3707,7 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="92"/>
+      <c r="A10" s="99"/>
       <c r="B10" s="89"/>
       <c r="C10" s="13" t="s">
         <v>188</v>
@@ -3721,13 +3721,13 @@
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="92"/>
+      <c r="A11" s="99"/>
       <c r="B11" s="89"/>
       <c r="E11" s="33"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="92"/>
-      <c r="B12" s="94" t="s">
+      <c r="A12" s="99"/>
+      <c r="B12" s="107" t="s">
         <v>364</v>
       </c>
       <c r="C12" s="35" t="s">
@@ -3742,8 +3742,8 @@
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="92"/>
-      <c r="B13" s="95"/>
+      <c r="A13" s="99"/>
+      <c r="B13" s="97"/>
       <c r="C13" s="13" t="s">
         <v>363</v>
       </c>
@@ -3756,8 +3756,8 @@
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="92"/>
-      <c r="B14" s="95"/>
+      <c r="A14" s="99"/>
+      <c r="B14" s="97"/>
       <c r="C14" s="13" t="s">
         <v>380</v>
       </c>
@@ -3770,8 +3770,8 @@
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="92"/>
-      <c r="B15" s="95"/>
+      <c r="A15" s="99"/>
+      <c r="B15" s="97"/>
       <c r="C15" s="13" t="s">
         <v>139</v>
       </c>
@@ -3784,8 +3784,8 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="92"/>
-      <c r="B16" s="95"/>
+      <c r="A16" s="99"/>
+      <c r="B16" s="97"/>
       <c r="C16" s="13" t="s">
         <v>238</v>
       </c>
@@ -3798,8 +3798,8 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="92"/>
-      <c r="B17" s="95"/>
+      <c r="A17" s="99"/>
+      <c r="B17" s="97"/>
       <c r="C17" s="13" t="s">
         <v>84</v>
       </c>
@@ -3812,8 +3812,8 @@
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="92"/>
-      <c r="B18" s="95"/>
+      <c r="A18" s="99"/>
+      <c r="B18" s="97"/>
       <c r="C18" s="13" t="s">
         <v>141</v>
       </c>
@@ -3826,8 +3826,8 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="92"/>
-      <c r="B19" s="95"/>
+      <c r="A19" s="99"/>
+      <c r="B19" s="97"/>
       <c r="C19" s="13" t="s">
         <v>155</v>
       </c>
@@ -3840,8 +3840,8 @@
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="92"/>
-      <c r="B20" s="95"/>
+      <c r="A20" s="99"/>
+      <c r="B20" s="97"/>
       <c r="C20" s="13" t="s">
         <v>196</v>
       </c>
@@ -3854,8 +3854,8 @@
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="92"/>
-      <c r="B21" s="95"/>
+      <c r="A21" s="99"/>
+      <c r="B21" s="97"/>
       <c r="C21" s="13" t="s">
         <v>167</v>
       </c>
@@ -3868,8 +3868,8 @@
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="92"/>
-      <c r="B22" s="95"/>
+      <c r="A22" s="99"/>
+      <c r="B22" s="97"/>
       <c r="C22" s="13" t="s">
         <v>188</v>
       </c>
@@ -3882,15 +3882,15 @@
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="92"/>
-      <c r="B23" s="96"/>
+      <c r="A23" s="99"/>
+      <c r="B23" s="108"/>
       <c r="C23" s="36"/>
       <c r="D23" s="36"/>
       <c r="E23" s="37"/>
       <c r="F23" s="36"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="92"/>
+      <c r="A24" s="99"/>
       <c r="B24" s="88" t="s">
         <v>262</v>
       </c>
@@ -3906,7 +3906,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="92"/>
+      <c r="A25" s="99"/>
       <c r="B25" s="89"/>
       <c r="C25" s="13" t="s">
         <v>107</v>
@@ -3920,7 +3920,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="92"/>
+      <c r="A26" s="99"/>
       <c r="B26" s="89"/>
       <c r="C26" s="13" t="s">
         <v>84</v>
@@ -3934,7 +3934,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="92"/>
+      <c r="A27" s="99"/>
       <c r="B27" s="89"/>
       <c r="C27" s="13" t="s">
         <v>283</v>
@@ -3948,7 +3948,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="92"/>
+      <c r="A28" s="99"/>
       <c r="B28" s="89"/>
       <c r="C28" s="13" t="s">
         <v>141</v>
@@ -3962,7 +3962,7 @@
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="92"/>
+      <c r="A29" s="99"/>
       <c r="B29" s="89"/>
       <c r="C29" s="13" t="s">
         <v>155</v>
@@ -3976,7 +3976,7 @@
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="92"/>
+      <c r="A30" s="99"/>
       <c r="B30" s="89"/>
       <c r="C30" s="13" t="s">
         <v>196</v>
@@ -3990,7 +3990,7 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="92"/>
+      <c r="A31" s="99"/>
       <c r="B31" s="89"/>
       <c r="C31" s="13" t="s">
         <v>167</v>
@@ -4004,7 +4004,7 @@
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="92"/>
+      <c r="A32" s="99"/>
       <c r="B32" s="89"/>
       <c r="C32" s="13" t="s">
         <v>188</v>
@@ -4018,7 +4018,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="92"/>
+      <c r="A33" s="99"/>
       <c r="B33" s="90"/>
       <c r="C33" s="36"/>
       <c r="D33" s="36"/>
@@ -4026,7 +4026,7 @@
       <c r="F33" s="36"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="92"/>
+      <c r="A34" s="99"/>
       <c r="B34" s="87" t="s">
         <v>229</v>
       </c>
@@ -4042,7 +4042,7 @@
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="92"/>
+      <c r="A35" s="99"/>
       <c r="B35" s="87"/>
       <c r="C35" s="13" t="s">
         <v>107</v>
@@ -4056,7 +4056,7 @@
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="92"/>
+      <c r="A36" s="99"/>
       <c r="B36" s="87"/>
       <c r="C36" s="13" t="s">
         <v>84</v>
@@ -4070,7 +4070,7 @@
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="92"/>
+      <c r="A37" s="99"/>
       <c r="B37" s="87"/>
       <c r="C37" s="13" t="s">
         <v>270</v>
@@ -4084,7 +4084,7 @@
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="92"/>
+      <c r="A38" s="99"/>
       <c r="B38" s="87"/>
       <c r="C38" s="13" t="s">
         <v>248</v>
@@ -4098,7 +4098,7 @@
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="92"/>
+      <c r="A39" s="99"/>
       <c r="B39" s="87"/>
       <c r="C39" s="13" t="s">
         <v>141</v>
@@ -4112,7 +4112,7 @@
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="92"/>
+      <c r="A40" s="99"/>
       <c r="B40" s="87"/>
       <c r="C40" s="13" t="s">
         <v>155</v>
@@ -4126,7 +4126,7 @@
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="92"/>
+      <c r="A41" s="99"/>
       <c r="B41" s="87"/>
       <c r="C41" s="13" t="s">
         <v>196</v>
@@ -4140,7 +4140,7 @@
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="92"/>
+      <c r="A42" s="99"/>
       <c r="B42" s="87"/>
       <c r="C42" s="13" t="s">
         <v>167</v>
@@ -4154,7 +4154,7 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="92"/>
+      <c r="A43" s="99"/>
       <c r="B43" s="87"/>
       <c r="C43" s="13" t="s">
         <v>188</v>
@@ -4168,15 +4168,15 @@
       </c>
     </row>
     <row r="44" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="92"/>
+      <c r="A44" s="99"/>
       <c r="B44" s="87"/>
       <c r="E44" s="33"/>
     </row>
     <row r="45" spans="1:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="91" t="s">
+      <c r="A45" s="93" t="s">
         <v>71</v>
       </c>
-      <c r="B45" s="100" t="s">
+      <c r="B45" s="110" t="s">
         <v>3</v>
       </c>
       <c r="C45" s="26" t="s">
@@ -4191,7 +4191,7 @@
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A46" s="92"/>
+      <c r="A46" s="99"/>
       <c r="B46" s="87"/>
       <c r="C46" s="13" t="s">
         <v>111</v>
@@ -4205,7 +4205,7 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A47" s="92"/>
+      <c r="A47" s="99"/>
       <c r="B47" s="87"/>
       <c r="C47" s="13" t="s">
         <v>135</v>
@@ -4219,7 +4219,7 @@
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A48" s="92"/>
+      <c r="A48" s="99"/>
       <c r="B48" s="87"/>
       <c r="C48" s="13" t="s">
         <v>136</v>
@@ -4233,7 +4233,7 @@
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A49" s="92"/>
+      <c r="A49" s="99"/>
       <c r="B49" s="87"/>
       <c r="C49" s="13" t="s">
         <v>141</v>
@@ -4247,7 +4247,7 @@
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A50" s="92"/>
+      <c r="A50" s="99"/>
       <c r="B50" s="87"/>
       <c r="C50" s="13" t="s">
         <v>155</v>
@@ -4261,7 +4261,7 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A51" s="92"/>
+      <c r="A51" s="99"/>
       <c r="B51" s="87"/>
       <c r="C51" s="13" t="s">
         <v>196</v>
@@ -4275,7 +4275,7 @@
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A52" s="92"/>
+      <c r="A52" s="99"/>
       <c r="B52" s="87"/>
       <c r="C52" s="13" t="s">
         <v>167</v>
@@ -4289,7 +4289,7 @@
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A53" s="92"/>
+      <c r="A53" s="99"/>
       <c r="B53" s="87"/>
       <c r="C53" s="13" t="s">
         <v>188</v>
@@ -4303,15 +4303,15 @@
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A54" s="92"/>
-      <c r="B54" s="101"/>
+      <c r="A54" s="99"/>
+      <c r="B54" s="102"/>
       <c r="C54" s="36"/>
       <c r="D54" s="36"/>
       <c r="E54" s="37"/>
       <c r="F54" s="36"/>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A55" s="92"/>
+      <c r="A55" s="99"/>
       <c r="B55" s="87" t="s">
         <v>305</v>
       </c>
@@ -4327,7 +4327,7 @@
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A56" s="92"/>
+      <c r="A56" s="99"/>
       <c r="B56" s="87"/>
       <c r="C56" s="13" t="s">
         <v>111</v>
@@ -4341,7 +4341,7 @@
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A57" s="92"/>
+      <c r="A57" s="99"/>
       <c r="B57" s="87"/>
       <c r="C57" s="13" t="s">
         <v>135</v>
@@ -4355,7 +4355,7 @@
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A58" s="92"/>
+      <c r="A58" s="99"/>
       <c r="B58" s="87"/>
       <c r="C58" s="13" t="s">
         <v>136</v>
@@ -4369,7 +4369,7 @@
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A59" s="92"/>
+      <c r="A59" s="99"/>
       <c r="B59" s="87"/>
       <c r="C59" s="13" t="s">
         <v>141</v>
@@ -4383,7 +4383,7 @@
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A60" s="92"/>
+      <c r="A60" s="99"/>
       <c r="B60" s="87"/>
       <c r="C60" s="13" t="s">
         <v>155</v>
@@ -4397,7 +4397,7 @@
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A61" s="92"/>
+      <c r="A61" s="99"/>
       <c r="B61" s="87"/>
       <c r="C61" s="13" t="s">
         <v>196</v>
@@ -4411,7 +4411,7 @@
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A62" s="92"/>
+      <c r="A62" s="99"/>
       <c r="B62" s="87"/>
       <c r="C62" s="13" t="s">
         <v>167</v>
@@ -4425,7 +4425,7 @@
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A63" s="92"/>
+      <c r="A63" s="99"/>
       <c r="B63" s="87"/>
       <c r="C63" s="13" t="s">
         <v>188</v>
@@ -4439,13 +4439,13 @@
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A64" s="92"/>
-      <c r="B64" s="101"/>
+      <c r="A64" s="99"/>
+      <c r="B64" s="102"/>
       <c r="E64" s="33"/>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="92"/>
-      <c r="B65" s="98" t="s">
+      <c r="A65" s="99"/>
+      <c r="B65" s="101" t="s">
         <v>6</v>
       </c>
       <c r="C65" s="35" t="s">
@@ -4460,7 +4460,7 @@
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="92"/>
+      <c r="A66" s="99"/>
       <c r="B66" s="87"/>
       <c r="C66" s="13" t="s">
         <v>113</v>
@@ -4474,7 +4474,7 @@
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="92"/>
+      <c r="A67" s="99"/>
       <c r="B67" s="89"/>
       <c r="C67" s="13" t="s">
         <v>111</v>
@@ -4488,7 +4488,7 @@
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="92"/>
+      <c r="A68" s="99"/>
       <c r="B68" s="89"/>
       <c r="C68" s="13" t="s">
         <v>107</v>
@@ -4502,7 +4502,7 @@
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="92"/>
+      <c r="A69" s="99"/>
       <c r="B69" s="89"/>
       <c r="C69" s="13" t="s">
         <v>126</v>
@@ -4516,7 +4516,7 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="92"/>
+      <c r="A70" s="99"/>
       <c r="B70" s="89"/>
       <c r="C70" s="13" t="s">
         <v>127</v>
@@ -4530,7 +4530,7 @@
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="92"/>
+      <c r="A71" s="99"/>
       <c r="B71" s="89"/>
       <c r="C71" s="13" t="s">
         <v>141</v>
@@ -4544,7 +4544,7 @@
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="92"/>
+      <c r="A72" s="99"/>
       <c r="B72" s="89"/>
       <c r="C72" s="13" t="s">
         <v>155</v>
@@ -4558,7 +4558,7 @@
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="92"/>
+      <c r="A73" s="99"/>
       <c r="B73" s="89"/>
       <c r="C73" s="13" t="s">
         <v>196</v>
@@ -4572,7 +4572,7 @@
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="92"/>
+      <c r="A74" s="99"/>
       <c r="B74" s="89"/>
       <c r="C74" s="13" t="s">
         <v>167</v>
@@ -4586,7 +4586,7 @@
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="92"/>
+      <c r="A75" s="99"/>
       <c r="B75" s="89"/>
       <c r="C75" s="13" t="s">
         <v>188</v>
@@ -4600,18 +4600,18 @@
       </c>
     </row>
     <row r="76" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="97"/>
-      <c r="B76" s="99"/>
+      <c r="A76" s="100"/>
+      <c r="B76" s="109"/>
       <c r="C76" s="40"/>
       <c r="D76" s="40"/>
       <c r="E76" s="41"/>
       <c r="F76" s="40"/>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="91" t="s">
+      <c r="A77" s="93" t="s">
         <v>72</v>
       </c>
-      <c r="B77" s="93" t="s">
+      <c r="B77" s="95" t="s">
         <v>73</v>
       </c>
       <c r="C77" s="26" t="s">
@@ -4626,7 +4626,7 @@
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="92"/>
+      <c r="A78" s="99"/>
       <c r="B78" s="89"/>
       <c r="C78" s="13" t="s">
         <v>153</v>
@@ -4640,13 +4640,13 @@
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="92"/>
+      <c r="A79" s="99"/>
       <c r="B79" s="90"/>
       <c r="E79" s="31"/>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="92"/>
-      <c r="B80" s="98" t="s">
+      <c r="A80" s="99"/>
+      <c r="B80" s="101" t="s">
         <v>4</v>
       </c>
       <c r="C80" s="35" t="s">
@@ -4661,7 +4661,7 @@
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A81" s="92"/>
+      <c r="A81" s="99"/>
       <c r="B81" s="87"/>
       <c r="C81" s="13" t="s">
         <v>107</v>
@@ -4675,7 +4675,7 @@
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A82" s="92"/>
+      <c r="A82" s="99"/>
       <c r="B82" s="87"/>
       <c r="C82" s="13" t="s">
         <v>122</v>
@@ -4689,7 +4689,7 @@
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A83" s="92"/>
+      <c r="A83" s="99"/>
       <c r="B83" s="87"/>
       <c r="C83" s="13" t="s">
         <v>141</v>
@@ -4703,7 +4703,7 @@
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A84" s="92"/>
+      <c r="A84" s="99"/>
       <c r="B84" s="87"/>
       <c r="C84" s="13" t="s">
         <v>155</v>
@@ -4717,7 +4717,7 @@
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A85" s="92"/>
+      <c r="A85" s="99"/>
       <c r="B85" s="87"/>
       <c r="C85" s="13" t="s">
         <v>161</v>
@@ -4731,7 +4731,7 @@
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A86" s="92"/>
+      <c r="A86" s="99"/>
       <c r="B86" s="87"/>
       <c r="C86" s="13" t="s">
         <v>196</v>
@@ -4745,7 +4745,7 @@
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A87" s="92"/>
+      <c r="A87" s="99"/>
       <c r="B87" s="87"/>
       <c r="C87" s="13" t="s">
         <v>167</v>
@@ -4759,7 +4759,7 @@
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A88" s="92"/>
+      <c r="A88" s="99"/>
       <c r="B88" s="87"/>
       <c r="C88" s="13" t="s">
         <v>188</v>
@@ -4773,12 +4773,12 @@
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A89" s="92"/>
-      <c r="B89" s="101"/>
+      <c r="A89" s="99"/>
+      <c r="B89" s="102"/>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A90" s="92"/>
-      <c r="B90" s="98" t="s">
+      <c r="A90" s="99"/>
+      <c r="B90" s="101" t="s">
         <v>5</v>
       </c>
       <c r="C90" s="35" t="s">
@@ -4793,7 +4793,7 @@
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A91" s="92"/>
+      <c r="A91" s="99"/>
       <c r="B91" s="87"/>
       <c r="C91" s="13" t="s">
         <v>108</v>
@@ -4807,7 +4807,7 @@
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A92" s="92"/>
+      <c r="A92" s="99"/>
       <c r="B92" s="87"/>
       <c r="C92" s="13" t="s">
         <v>120</v>
@@ -4821,7 +4821,7 @@
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A93" s="92"/>
+      <c r="A93" s="99"/>
       <c r="B93" s="87"/>
       <c r="C93" s="13" t="s">
         <v>141</v>
@@ -4835,7 +4835,7 @@
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" s="92"/>
+      <c r="A94" s="99"/>
       <c r="B94" s="87"/>
       <c r="C94" s="13" t="s">
         <v>155</v>
@@ -4849,7 +4849,7 @@
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A95" s="92"/>
+      <c r="A95" s="99"/>
       <c r="B95" s="87"/>
       <c r="C95" s="13" t="s">
         <v>161</v>
@@ -4863,7 +4863,7 @@
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" s="92"/>
+      <c r="A96" s="99"/>
       <c r="B96" s="87"/>
       <c r="C96" s="13" t="s">
         <v>196</v>
@@ -4877,7 +4877,7 @@
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A97" s="92"/>
+      <c r="A97" s="99"/>
       <c r="B97" s="87"/>
       <c r="C97" s="13" t="s">
         <v>167</v>
@@ -4891,7 +4891,7 @@
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A98" s="92"/>
+      <c r="A98" s="99"/>
       <c r="B98" s="87"/>
       <c r="C98" s="13" t="s">
         <v>188</v>
@@ -4905,14 +4905,14 @@
       </c>
     </row>
     <row r="99" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="97"/>
-      <c r="B99" s="104"/>
+      <c r="A99" s="100"/>
+      <c r="B99" s="103"/>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A100" s="91" t="s">
+      <c r="A100" s="93" t="s">
         <v>76</v>
       </c>
-      <c r="B100" s="93" t="s">
+      <c r="B100" s="95" t="s">
         <v>73</v>
       </c>
       <c r="C100" s="26" t="s">
@@ -4927,7 +4927,7 @@
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A101" s="92"/>
+      <c r="A101" s="99"/>
       <c r="B101" s="89"/>
       <c r="C101" s="13" t="s">
         <v>228</v>
@@ -4941,7 +4941,7 @@
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A102" s="92"/>
+      <c r="A102" s="99"/>
       <c r="B102" s="89"/>
       <c r="C102" s="13" t="s">
         <v>150</v>
@@ -4955,7 +4955,7 @@
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A103" s="92"/>
+      <c r="A103" s="99"/>
       <c r="B103" s="90"/>
       <c r="C103" s="36"/>
       <c r="D103" s="36"/>
@@ -4963,7 +4963,7 @@
       <c r="F103" s="36"/>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A104" s="92"/>
+      <c r="A104" s="99"/>
       <c r="B104" s="88" t="s">
         <v>292</v>
       </c>
@@ -4979,7 +4979,7 @@
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A105" s="92"/>
+      <c r="A105" s="99"/>
       <c r="B105" s="89"/>
       <c r="C105" s="13" t="s">
         <v>297</v>
@@ -4993,7 +4993,7 @@
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A106" s="92"/>
+      <c r="A106" s="99"/>
       <c r="B106" s="89"/>
       <c r="C106" s="13" t="s">
         <v>298</v>
@@ -5007,12 +5007,12 @@
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A107" s="92"/>
+      <c r="A107" s="99"/>
       <c r="B107" s="90"/>
       <c r="E107" s="33"/>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A108" s="92"/>
+      <c r="A108" s="99"/>
       <c r="B108" s="88" t="s">
         <v>79</v>
       </c>
@@ -5028,8 +5028,8 @@
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A109" s="92"/>
-      <c r="B109" s="105"/>
+      <c r="A109" s="99"/>
+      <c r="B109" s="91"/>
       <c r="C109" s="70" t="s">
         <v>151</v>
       </c>
@@ -5042,7 +5042,7 @@
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A110" s="92"/>
+      <c r="A110" s="99"/>
       <c r="B110" s="90"/>
       <c r="C110" s="36"/>
       <c r="D110" s="36"/>
@@ -5050,8 +5050,8 @@
       <c r="F110" s="36"/>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A111" s="92"/>
-      <c r="B111" s="106" t="s">
+      <c r="A111" s="99"/>
+      <c r="B111" s="104" t="s">
         <v>371</v>
       </c>
       <c r="C111" s="35" t="s">
@@ -5066,8 +5066,8 @@
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A112" s="92"/>
-      <c r="B112" s="107"/>
+      <c r="A112" s="99"/>
+      <c r="B112" s="105"/>
       <c r="C112" s="70" t="s">
         <v>376</v>
       </c>
@@ -5080,16 +5080,16 @@
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A113" s="92"/>
-      <c r="B113" s="108"/>
+      <c r="A113" s="99"/>
+      <c r="B113" s="106"/>
       <c r="C113" s="36"/>
       <c r="D113" s="36"/>
       <c r="E113" s="37"/>
       <c r="F113" s="36"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A114" s="92"/>
-      <c r="B114" s="102" t="s">
+      <c r="A114" s="99"/>
+      <c r="B114" s="96" t="s">
         <v>331</v>
       </c>
       <c r="C114" s="13" t="s">
@@ -5104,8 +5104,8 @@
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A115" s="92"/>
-      <c r="B115" s="95"/>
+      <c r="A115" s="99"/>
+      <c r="B115" s="97"/>
       <c r="C115" s="13" t="s">
         <v>362</v>
       </c>
@@ -5118,18 +5118,18 @@
       </c>
     </row>
     <row r="116" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A116" s="97"/>
-      <c r="B116" s="103"/>
+      <c r="A116" s="100"/>
+      <c r="B116" s="98"/>
       <c r="C116" s="40"/>
       <c r="D116" s="40"/>
       <c r="E116" s="41"/>
       <c r="F116" s="40"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A117" s="91" t="s">
+      <c r="A117" s="93" t="s">
         <v>163</v>
       </c>
-      <c r="B117" s="93" t="s">
+      <c r="B117" s="95" t="s">
         <v>13</v>
       </c>
       <c r="C117" s="26" t="s">
@@ -5144,8 +5144,8 @@
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A118" s="110"/>
-      <c r="B118" s="105"/>
+      <c r="A118" s="94"/>
+      <c r="B118" s="91"/>
       <c r="C118" s="13" t="s">
         <v>174</v>
       </c>
@@ -5157,7 +5157,7 @@
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="110"/>
+      <c r="A119" s="94"/>
       <c r="B119" s="90"/>
       <c r="C119" s="36"/>
       <c r="D119" s="36"/>
@@ -5165,7 +5165,7 @@
       <c r="F119" s="36"/>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="110"/>
+      <c r="A120" s="94"/>
       <c r="B120" s="88" t="s">
         <v>183</v>
       </c>
@@ -5180,8 +5180,8 @@
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="110"/>
-      <c r="B121" s="105"/>
+      <c r="A121" s="94"/>
+      <c r="B121" s="91"/>
       <c r="C121" s="13" t="s">
         <v>181</v>
       </c>
@@ -5193,8 +5193,8 @@
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="110"/>
-      <c r="B122" s="105"/>
+      <c r="A122" s="94"/>
+      <c r="B122" s="91"/>
       <c r="C122" s="13" t="s">
         <v>177</v>
       </c>
@@ -5206,8 +5206,8 @@
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" s="110"/>
-      <c r="B123" s="105"/>
+      <c r="A123" s="94"/>
+      <c r="B123" s="91"/>
       <c r="C123" s="13" t="s">
         <v>179</v>
       </c>
@@ -5219,8 +5219,8 @@
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="110"/>
-      <c r="B124" s="105"/>
+      <c r="A124" s="94"/>
+      <c r="B124" s="91"/>
       <c r="C124" s="13" t="s">
         <v>182</v>
       </c>
@@ -5232,8 +5232,8 @@
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" s="110"/>
-      <c r="B125" s="105"/>
+      <c r="A125" s="94"/>
+      <c r="B125" s="91"/>
       <c r="C125" s="13" t="s">
         <v>191</v>
       </c>
@@ -5245,11 +5245,11 @@
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="110"/>
+      <c r="A126" s="94"/>
       <c r="B126" s="90"/>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="110"/>
+      <c r="A127" s="94"/>
       <c r="B127" s="88" t="s">
         <v>206</v>
       </c>
@@ -5265,8 +5265,8 @@
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="110"/>
-      <c r="B128" s="105"/>
+      <c r="A128" s="94"/>
+      <c r="B128" s="91"/>
       <c r="C128" s="13" t="s">
         <v>204</v>
       </c>
@@ -5278,8 +5278,8 @@
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="110"/>
-      <c r="B129" s="105"/>
+      <c r="A129" s="94"/>
+      <c r="B129" s="91"/>
       <c r="C129" s="13" t="s">
         <v>215</v>
       </c>
@@ -5291,8 +5291,8 @@
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="110"/>
-      <c r="B130" s="105"/>
+      <c r="A130" s="94"/>
+      <c r="B130" s="91"/>
       <c r="C130" s="13" t="s">
         <v>205</v>
       </c>
@@ -5304,8 +5304,8 @@
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="110"/>
-      <c r="B131" s="105"/>
+      <c r="A131" s="94"/>
+      <c r="B131" s="91"/>
       <c r="C131" s="13" t="s">
         <v>300</v>
       </c>
@@ -5317,8 +5317,8 @@
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="110"/>
-      <c r="B132" s="105"/>
+      <c r="A132" s="94"/>
+      <c r="B132" s="91"/>
       <c r="C132" s="44" t="s">
         <v>324</v>
       </c>
@@ -5331,8 +5331,8 @@
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="110"/>
-      <c r="B133" s="105"/>
+      <c r="A133" s="94"/>
+      <c r="B133" s="91"/>
       <c r="C133" s="44" t="s">
         <v>326</v>
       </c>
@@ -5345,8 +5345,8 @@
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="110"/>
-      <c r="B134" s="105"/>
+      <c r="A134" s="94"/>
+      <c r="B134" s="91"/>
       <c r="C134" s="13" t="s">
         <v>217</v>
       </c>
@@ -5358,8 +5358,8 @@
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="110"/>
-      <c r="B135" s="105"/>
+      <c r="A135" s="94"/>
+      <c r="B135" s="91"/>
       <c r="C135" s="13" t="s">
         <v>221</v>
       </c>
@@ -5371,8 +5371,8 @@
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="110"/>
-      <c r="B136" s="105"/>
+      <c r="A136" s="94"/>
+      <c r="B136" s="91"/>
       <c r="C136" s="13" t="s">
         <v>202</v>
       </c>
@@ -5384,8 +5384,8 @@
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A137" s="110"/>
-      <c r="B137" s="105"/>
+      <c r="A137" s="94"/>
+      <c r="B137" s="91"/>
       <c r="C137" s="44" t="s">
         <v>249</v>
       </c>
@@ -5398,8 +5398,8 @@
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" s="110"/>
-      <c r="B138" s="105"/>
+      <c r="A138" s="94"/>
+      <c r="B138" s="91"/>
       <c r="C138" s="44" t="s">
         <v>383</v>
       </c>
@@ -5412,8 +5412,8 @@
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="110"/>
-      <c r="B139" s="105"/>
+      <c r="A139" s="94"/>
+      <c r="B139" s="91"/>
       <c r="C139" s="44" t="s">
         <v>365</v>
       </c>
@@ -5426,8 +5426,8 @@
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" s="110"/>
-      <c r="B140" s="105"/>
+      <c r="A140" s="94"/>
+      <c r="B140" s="91"/>
       <c r="C140" s="44" t="s">
         <v>385</v>
       </c>
@@ -5440,7 +5440,7 @@
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A141" s="110"/>
+      <c r="A141" s="94"/>
       <c r="B141" s="90"/>
       <c r="C141" s="44"/>
       <c r="D141" s="44"/>
@@ -5448,7 +5448,7 @@
       <c r="F141" s="44"/>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A142" s="110"/>
+      <c r="A142" s="94"/>
       <c r="B142" s="88" t="s">
         <v>222</v>
       </c>
@@ -5464,8 +5464,8 @@
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A143" s="110"/>
-      <c r="B143" s="105"/>
+      <c r="A143" s="94"/>
+      <c r="B143" s="91"/>
       <c r="C143" s="70" t="s">
         <v>302</v>
       </c>
@@ -5478,8 +5478,8 @@
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" s="110"/>
-      <c r="B144" s="105"/>
+      <c r="A144" s="94"/>
+      <c r="B144" s="91"/>
       <c r="C144" s="70" t="s">
         <v>225</v>
       </c>
@@ -5492,8 +5492,8 @@
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A145" s="110"/>
-      <c r="B145" s="105"/>
+      <c r="A145" s="94"/>
+      <c r="B145" s="91"/>
       <c r="C145" s="72" t="s">
         <v>251</v>
       </c>
@@ -5506,8 +5506,8 @@
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A146" s="110"/>
-      <c r="B146" s="105"/>
+      <c r="A146" s="94"/>
+      <c r="B146" s="91"/>
       <c r="C146" s="72" t="s">
         <v>366</v>
       </c>
@@ -5520,7 +5520,7 @@
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A147" s="110"/>
+      <c r="A147" s="94"/>
       <c r="B147" s="90"/>
       <c r="C147" s="36"/>
       <c r="D147" s="36"/>
@@ -5528,8 +5528,8 @@
       <c r="F147" s="36"/>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A148" s="110"/>
-      <c r="B148" s="109" t="s">
+      <c r="A148" s="94"/>
+      <c r="B148" s="92" t="s">
         <v>386</v>
       </c>
       <c r="C148" s="70" t="s">
@@ -5544,8 +5544,8 @@
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A149" s="110"/>
-      <c r="B149" s="109"/>
+      <c r="A149" s="94"/>
+      <c r="B149" s="92"/>
       <c r="C149" s="70" t="s">
         <v>388</v>
       </c>
@@ -5565,12 +5565,15 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B142:B147"/>
-    <mergeCell ref="B148:B149"/>
-    <mergeCell ref="A117:A149"/>
-    <mergeCell ref="B117:B119"/>
-    <mergeCell ref="B127:B141"/>
-    <mergeCell ref="B120:B126"/>
+    <mergeCell ref="A2:A44"/>
+    <mergeCell ref="B2:B11"/>
+    <mergeCell ref="B12:B23"/>
+    <mergeCell ref="B34:B44"/>
+    <mergeCell ref="A45:A76"/>
+    <mergeCell ref="B65:B76"/>
+    <mergeCell ref="B24:B33"/>
+    <mergeCell ref="B45:B54"/>
+    <mergeCell ref="B55:B64"/>
     <mergeCell ref="B114:B116"/>
     <mergeCell ref="B77:B79"/>
     <mergeCell ref="A77:A99"/>
@@ -5581,15 +5584,12 @@
     <mergeCell ref="B104:B107"/>
     <mergeCell ref="B108:B110"/>
     <mergeCell ref="B111:B113"/>
-    <mergeCell ref="A2:A44"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="B12:B23"/>
-    <mergeCell ref="B34:B44"/>
-    <mergeCell ref="A45:A76"/>
-    <mergeCell ref="B65:B76"/>
-    <mergeCell ref="B24:B33"/>
-    <mergeCell ref="B45:B54"/>
-    <mergeCell ref="B55:B64"/>
+    <mergeCell ref="B142:B147"/>
+    <mergeCell ref="B148:B149"/>
+    <mergeCell ref="A117:A149"/>
+    <mergeCell ref="B117:B119"/>
+    <mergeCell ref="B127:B141"/>
+    <mergeCell ref="B120:B126"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>